<commit_message>
Fix inventory reset import with Gemini slots
</commit_message>
<xml_diff>
--- a/imports/import_CHATGPT_ONLY_READY1.xlsx
+++ b/imports/import_CHATGPT_ONLY_READY1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\telegram-auto-sell-bot\imports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5199BD65-2D63-4ACE-8350-97E554D19D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1C20F7B8-59AE-4804-A25B-E438C0A985BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>